<commit_message>
2.6 Array Formulas Completed
</commit_message>
<xml_diff>
--- a/2_Formulas_Functions/3_Logical_Functions.xlsx
+++ b/2_Formulas_Functions/3_Logical_Functions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nazil\1 A CHARUSAT\1 Visual Studio Code\Personal\DOA\1_Excel_DOA_Course\Excel_Data_Analytics_Course\2_Formulas_Functions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8063926F-B2A1-472D-9C76-ECB79527680F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06354CF7-9577-496A-9D29-1A421BCFC82F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{8CC555B5-3E06-43B6-9E5B-C0A1D3498DA4}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{8CC555B5-3E06-43B6-9E5B-C0A1D3498DA4}"/>
   </bookViews>
   <sheets>
     <sheet name="Data_1" sheetId="7" r:id="rId1"/>

</xml_diff>